<commit_message>
add "Last contacted" to contacts
</commit_message>
<xml_diff>
--- a/src/xlsx/fixtures/base-tracker.generated.xlsx
+++ b/src/xlsx/fixtures/base-tracker.generated.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="130">
   <si>
     <t>Pipeline summary</t>
   </si>
@@ -342,6 +342,9 @@
   </si>
   <si>
     <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Last contacted</t>
   </si>
   <si>
     <t>Maya Okafor</t>
@@ -1416,7 +1419,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1429,10 +1432,11 @@
     <col min="8" max="8" width="30" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
+    <col min="11" max="11" width="14" style="5" customWidth="1"/>
+    <col min="12" max="12" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>84</v>
       </c>
@@ -1463,11 +1467,14 @@
       <c r="J1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1475,34 +1482,37 @@
         <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
         <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J2" t="s">
-        <v>99</v>
-      </c>
-      <c r="K2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K2" s="5">
+        <v>46287</v>
+      </c>
+      <c r="L2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1510,22 +1520,23 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -1533,28 +1544,31 @@
         <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
         <v>74</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="K4" s="5">
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -1562,28 +1576,29 @@
         <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E5" t="s">
         <v>74</v>
       </c>
       <c r="G5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I5" t="s">
-        <v>115</v>
-      </c>
-      <c r="K5" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K5" s="5"/>
+      <c r="L5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -1591,19 +1606,20 @@
         <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="K6" s="5"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -1611,22 +1627,23 @@
         <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E7" t="s">
         <v>74</v>
       </c>
       <c r="G7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -1634,26 +1651,29 @@
         <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E8" t="s">
         <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I8" t="s">
-        <v>128</v>
+        <v>129</v>
+      </c>
+      <c r="K8" s="5">
+        <v>46295</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K8"/>
+  <autoFilter ref="A1:L8"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D2:D2000">
       <formula1>"Economic Buyer,Champion,Technical Buyer,End User,Influencer,Blocker,Gatekeeper,Channel"</formula1>

</xml_diff>

<commit_message>
Track replies on contacts, drop pipeline date stamping
Contacts get a required "Last reply" date beside "Last contacted", with
one-click "Replied today" / "Contacted today" buttons in the contact panel.
Changing a prospect's stage now only sets its status: Sent, Replied and
Last touch are no longer stamped, and Last touch is gone from the new and
Discovery layouts. "Needs follow-up" reads the contacts' dates instead.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/xlsx/fixtures/base-tracker.generated.xlsx
+++ b/src/xlsx/fixtures/base-tracker.generated.xlsx
@@ -125,9 +125,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Last touch</t>
-  </si>
-  <si>
     <t>Next step</t>
   </si>
   <si>
@@ -347,6 +344,9 @@
     <t>Last contacted</t>
   </si>
   <si>
+    <t>Last reply</t>
+  </si>
+  <si>
     <t>Maya Okafor</t>
   </si>
   <si>
@@ -460,8 +460,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="d mmm yyyy"/>
-    <numFmt numFmtId="165" formatCode="d mmm yyyy h:mm"/>
+    <numFmt numFmtId="164" formatCode="d mmm yyyy h:mm"/>
+    <numFmt numFmtId="165" formatCode="d mmm yyyy"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -524,16 +524,16 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,7 +1003,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <f>COUNTIF(Prospects!$R$2:$R$2000,"TRUE")</f>
+        <f>COUNTIF(Prospects!$Q$2:$Q$2000,"TRUE")</f>
         <v>1</v>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1040,82 +1040,78 @@
     <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="8" width="12" style="3" customWidth="1"/>
     <col min="9" max="9" width="18" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14" style="5" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
-    <col min="13" max="13" width="20" style="6" customWidth="1"/>
-    <col min="14" max="15" width="40" customWidth="1"/>
-    <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="44" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="36" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="20" style="5" customWidth="1"/>
+    <col min="13" max="14" width="40" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="44" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="R1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="S1" s="7" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -1124,13 +1120,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>35</v>
-      </c>
-      <c r="G2" t="s">
-        <v>36</v>
       </c>
       <c r="H2" s="3">
         <v>420</v>
@@ -1138,31 +1134,28 @@
       <c r="I2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="5">
-        <v>46287</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="J2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="5"/>
+      <c r="M2" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" t="s">
         <v>39</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="10"/>
+      <c r="R2" s="10"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="Q2" s="12"/>
-      <c r="S2" s="12"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>41</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -1171,13 +1164,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" t="s">
         <v>43</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>44</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
       </c>
       <c r="H3" s="3">
         <v>1100</v>
@@ -1185,31 +1178,28 @@
       <c r="I3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="5">
-        <v>46289</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" s="5"/>
+      <c r="M3" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="M3" s="6"/>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" t="s">
         <v>48</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="10"/>
+      <c r="R3" s="10"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
-      <c r="Q3" s="12"/>
-      <c r="S3" s="12"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
@@ -1218,13 +1208,13 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>53</v>
-      </c>
-      <c r="G4" t="s">
-        <v>54</v>
       </c>
       <c r="H4" s="3">
         <v>260</v>
@@ -1232,24 +1222,23 @@
       <c r="I4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="12" t="s">
+      <c r="L4" s="5"/>
+      <c r="M4" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="10"/>
+      <c r="O4" t="s">
         <v>55</v>
       </c>
-      <c r="O4" s="12"/>
-      <c r="P4" t="s">
+      <c r="P4" s="10"/>
+      <c r="R4" s="10"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>56</v>
       </c>
-      <c r="Q4" s="12"/>
-      <c r="S4" s="12"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -1258,13 +1247,13 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
         <v>59</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>60</v>
-      </c>
-      <c r="G5" t="s">
-        <v>61</v>
       </c>
       <c r="H5" s="3">
         <v>85</v>
@@ -1272,38 +1261,35 @@
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="5">
-        <v>46294</v>
+      <c r="J5" t="s">
+        <v>61</v>
       </c>
       <c r="K5" t="s">
         <v>62</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="5">
+        <v>46301.625</v>
+      </c>
+      <c r="M5" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="M5" s="6">
-        <v>46301.625</v>
-      </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="O5" s="12" t="s">
+      <c r="O5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q5" s="12" t="s">
+      <c r="R5" s="10"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>66</v>
       </c>
-      <c r="S5" s="12"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>67</v>
-      </c>
-      <c r="B6" t="s">
-        <v>68</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
@@ -1312,13 +1298,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" t="s">
         <v>69</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>70</v>
-      </c>
-      <c r="G6" t="s">
-        <v>71</v>
       </c>
       <c r="H6" s="3">
         <v>190</v>
@@ -1326,31 +1312,28 @@
       <c r="I6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="5">
-        <v>46275</v>
-      </c>
-      <c r="M6" s="6"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12" t="s">
+      <c r="L6" s="5"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" t="s">
         <v>72</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P6" s="10"/>
+      <c r="Q6" t="s">
         <v>73</v>
       </c>
-      <c r="Q6" s="12"/>
-      <c r="R6" t="s">
+      <c r="R6" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="S6" s="12" t="s">
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
@@ -1359,13 +1342,13 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>79</v>
-      </c>
-      <c r="G7" t="s">
-        <v>80</v>
       </c>
       <c r="H7" s="3">
         <v>60</v>
@@ -1373,30 +1356,27 @@
       <c r="I7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="5">
-        <v>46295</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="J7" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7" s="5"/>
+      <c r="M7" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="M7" s="6"/>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="10"/>
+      <c r="O7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" s="10"/>
+      <c r="R7" s="10"/>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="O7" s="12"/>
-      <c r="P7" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q7" s="12"/>
-      <c r="S7" s="12"/>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="13" t="s">
-        <v>83</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S7"/>
+  <autoFilter ref="A1:R7"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="C2:C2000">
       <formula1>"Direct,Aggregator"</formula1>
@@ -1404,7 +1384,7 @@
     <dataValidation type="list" allowBlank="1" sqref="I2:I2000">
       <formula1>"Not contacted,Contacted,Replied,Meeting booked,Proposal,Won,Dead"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="R2:R2000">
+    <dataValidation type="list" allowBlank="1" sqref="Q2:Q2000">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1419,7 +1399,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1432,54 +1412,58 @@
     <col min="8" max="8" width="30" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="14" style="5" customWidth="1"/>
-    <col min="12" max="12" width="40" customWidth="1"/>
+    <col min="11" max="11" width="14" style="12" customWidth="1"/>
+    <col min="12" max="12" width="12" style="12" customWidth="1"/>
+    <col min="13" max="13" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="L1" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>94</v>
@@ -1488,7 +1472,7 @@
         <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F2" t="s">
         <v>96</v>
@@ -1505,19 +1489,20 @@
       <c r="J2" t="s">
         <v>100</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="12">
         <v>46287</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="12"/>
+      <c r="M2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
         <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>33</v>
       </c>
       <c r="C3" t="s">
         <v>102</v>
@@ -1534,14 +1519,15 @@
       <c r="H3" t="s">
         <v>106</v>
       </c>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
         <v>41</v>
-      </c>
-      <c r="B4" t="s">
-        <v>42</v>
       </c>
       <c r="C4" t="s">
         <v>107</v>
@@ -1550,7 +1536,7 @@
         <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
         <v>109</v>
@@ -1564,16 +1550,19 @@
       <c r="J4" t="s">
         <v>112</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="12">
         <v>46290</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="12">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
       </c>
       <c r="C5" t="s">
         <v>113</v>
@@ -1582,7 +1571,7 @@
         <v>95</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
         <v>114</v>
@@ -1593,17 +1582,18 @@
       <c r="I5" t="s">
         <v>116</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" t="s">
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
         <v>57</v>
-      </c>
-      <c r="B6" t="s">
-        <v>58</v>
       </c>
       <c r="C6" t="s">
         <v>118</v>
@@ -1617,14 +1607,15 @@
       <c r="G6" t="s">
         <v>120</v>
       </c>
-      <c r="K6" s="5"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" t="s">
         <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
       </c>
       <c r="C7" t="s">
         <v>121</v>
@@ -1633,7 +1624,7 @@
         <v>122</v>
       </c>
       <c r="E7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
         <v>123</v>
@@ -1641,14 +1632,15 @@
       <c r="H7" t="s">
         <v>124</v>
       </c>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
         <v>76</v>
-      </c>
-      <c r="B8" t="s">
-        <v>77</v>
       </c>
       <c r="C8" t="s">
         <v>125</v>
@@ -1657,7 +1649,7 @@
         <v>126</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
         <v>127</v>
@@ -1668,12 +1660,13 @@
       <c r="I8" t="s">
         <v>129</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="12">
         <v>46295</v>
       </c>
+      <c r="L8" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:M8"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D2:D2000">
       <formula1>"Economic Buyer,Champion,Technical Buyer,End User,Influencer,Blocker,Gatekeeper,Channel"</formula1>

</xml_diff>

<commit_message>
Make Mudd's own columns always Mudd's
The columns Mudd relies on (Status, Company, ID, Intro message, the
meeting pair, Screened out and its reason; a contact's Name, Contact
type, Primary, Last contacted and Last reply) are found only by the
header Mudd writes, and on import take Mudd's header, type and dropdown
list whatever the sheet had; the cells are kept. The header aliases and
the type guesses that only served them are gone. The Columns dialog
lets these columns be hidden, not renamed, retyped or given other
options. The fixture's stages are now Mudd's, as the real tracker's are.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/xlsx/fixtures/base-tracker.generated.xlsx
+++ b/src/xlsx/fixtures/base-tracker.generated.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="131">
   <si>
     <t>Pipeline summary</t>
   </si>
@@ -80,10 +80,13 @@
     <t>Meeting booked</t>
   </si>
   <si>
-    <t>Proposal</t>
-  </si>
-  <si>
-    <t>Won</t>
+    <t>Clinic held</t>
+  </si>
+  <si>
+    <t>Trial</t>
+  </si>
+  <si>
+    <t>Signed</t>
   </si>
   <si>
     <t>Dead</t>
@@ -873,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -955,11 +958,11 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Proposal")*(Prospects!$C$2:$C$2000="Direct"))</f>
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Clinic held")*(Prospects!$C$2:$C$2000="Direct"))</f>
         <v>0</v>
       </c>
       <c r="C8">
-        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Proposal")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Clinic held")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
         <v>0</v>
       </c>
     </row>
@@ -968,11 +971,11 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Won")*(Prospects!$C$2:$C$2000="Direct"))</f>
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Trial")*(Prospects!$C$2:$C$2000="Direct"))</f>
         <v>0</v>
       </c>
       <c r="C9">
-        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Won")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Trial")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
         <v>0</v>
       </c>
     </row>
@@ -981,21 +984,25 @@
         <v>10</v>
       </c>
       <c r="B10">
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Signed")*(Prospects!$C$2:$C$2000="Direct"))</f>
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Signed")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
         <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Dead")*(Prospects!$C$2:$C$2000="Direct"))</f>
         <v>1</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <f>SUMPRODUCT((Prospects!$I$2:$I$2000="Dead")*(Prospects!$C$2:$C$2000="Aggregator"))</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <f>COUNTA(Prospects!$B$2:$B$2000)-1</f>
-        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -1003,8 +1010,8 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <f>COUNTIF(Prospects!$Q$2:$Q$2000,"TRUE")</f>
-        <v>1</v>
+        <f>COUNTA(Prospects!$B$2:$B$2000)-1</f>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1012,6 +1019,15 @@
         <v>13</v>
       </c>
       <c r="B14">
+        <f>COUNTIF(Prospects!$Q$2:$Q$2000,"TRUE")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
         <f>COUNTA(Contacts!$C$2:$C$2000)</f>
         <v>7</v>
       </c>
@@ -1052,66 +1068,66 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -1120,13 +1136,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H2" s="3">
         <v>420</v>
@@ -1135,27 +1151,27 @@
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P2" s="10"/>
       <c r="R2" s="10"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -1164,13 +1180,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" s="3">
         <v>1100</v>
@@ -1179,27 +1195,27 @@
         <v>6</v>
       </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P3" s="10"/>
       <c r="R3" s="10"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
@@ -1208,13 +1224,13 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H4" s="3">
         <v>260</v>
@@ -1224,21 +1240,21 @@
       </c>
       <c r="L4" s="5"/>
       <c r="M4" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N4" s="10"/>
       <c r="O4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P4" s="10"/>
       <c r="R4" s="10"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -1247,13 +1263,13 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H5" s="3">
         <v>85</v>
@@ -1262,34 +1278,34 @@
         <v>7</v>
       </c>
       <c r="J5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L5" s="5">
         <v>46301.625</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R5" s="10"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
@@ -1298,42 +1314,42 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H6" s="3">
         <v>190</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="10"/>
       <c r="N6" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P6" s="10"/>
       <c r="Q6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R6" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
@@ -1342,13 +1358,13 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H7" s="3">
         <v>60</v>
@@ -1357,22 +1373,22 @@
         <v>5</v>
       </c>
       <c r="J7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N7" s="10"/>
       <c r="O7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P7" s="10"/>
       <c r="R7" s="10"/>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1382,7 +1398,7 @@
       <formula1>"Direct,Aggregator"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="I2:I2000">
-      <formula1>"Not contacted,Contacted,Replied,Meeting booked,Proposal,Won,Dead"</formula1>
+      <formula1>"Not contacted,Contacted,Replied,Meeting booked,Clinic held,Trial,Signed,Dead"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="Q2:Q2000">
       <formula1>"TRUE,FALSE"</formula1>
@@ -1419,136 +1435,136 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K2" s="12">
         <v>46287</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K4" s="12">
         <v>46290</v>
@@ -1559,106 +1575,106 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K5" s="12"/>
       <c r="L5" s="12"/>
       <c r="M5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K8" s="12">
         <v>46295</v>

</xml_diff>

<commit_message>
Intro message per contact
Move the Intro message column from prospects to contacts: each contact
gets its own intro section (templates, Write with AI, Copy, Mark sent)
in its panel. Intro runs now take contact ids and write the draft to
that person. Draft intros works on selected contacts, or on each
selected prospect's contacts without an intro yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/xlsx/fixtures/base-tracker.generated.xlsx
+++ b/src/xlsx/fixtures/base-tracker.generated.xlsx
@@ -146,9 +146,6 @@
     <t>Source</t>
   </si>
   <si>
-    <t>Intro message</t>
-  </si>
-  <si>
     <t>Screened reason</t>
   </si>
   <si>
@@ -262,164 +259,167 @@
     <t>Office manager is the champion</t>
   </si>
   <si>
+    <t>P-005</t>
+  </si>
+  <si>
+    <t>Granite Peak Credit Union</t>
+  </si>
+  <si>
+    <t>Credit union</t>
+  </si>
+  <si>
+    <t>Boise, ID</t>
+  </si>
+  <si>
+    <t>granitepeakcu.example</t>
+  </si>
+  <si>
+    <t>Chose an incumbent</t>
+  </si>
+  <si>
+    <t>Conference</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Signed a three-year deal with another vendor</t>
+  </si>
+  <si>
+    <t>P-006</t>
+  </si>
+  <si>
+    <t>Saltmarsh Marine Supply</t>
+  </si>
+  <si>
+    <t>Distributor</t>
+  </si>
+  <si>
+    <t>Mobile, AL</t>
+  </si>
+  <si>
+    <t>saltmarshmarine.example</t>
+  </si>
+  <si>
+    <t>Call Thursday</t>
+  </si>
+  <si>
+    <t>Seasonal push before spring</t>
+  </si>
+  <si>
+    <t>Paste new rows directly above this line, columns already in this order.</t>
+  </si>
+  <si>
+    <t>Prospect ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Contact type</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Last contacted</t>
+  </si>
+  <si>
+    <t>Last reply</t>
+  </si>
+  <si>
+    <t>Intro message</t>
+  </si>
+  <si>
+    <t>Maya Okafor</t>
+  </si>
+  <si>
+    <t>Champion</t>
+  </si>
+  <si>
+    <t>Ms.</t>
+  </si>
+  <si>
+    <t>Plant Manager</t>
+  </si>
+  <si>
+    <t>maya.okafor@northwindfab.example</t>
+  </si>
+  <si>
+    <t>+1 937 555 0141</t>
+  </si>
+  <si>
+    <t>https://linkedin.example/in/maya-okafor</t>
+  </si>
+  <si>
+    <t>Met at the regional show</t>
+  </si>
+  <si>
+    <t>Tom Reyes</t>
+  </si>
+  <si>
+    <t>Technical Buyer</t>
+  </si>
+  <si>
+    <t>Mr.</t>
+  </si>
+  <si>
+    <t>IT Lead</t>
+  </si>
+  <si>
+    <t>tom.reyes@northwindfab.example</t>
+  </si>
+  <si>
+    <t>Priya Natarajan</t>
+  </si>
+  <si>
+    <t>Economic Buyer</t>
+  </si>
+  <si>
+    <t>VP Operations</t>
+  </si>
+  <si>
+    <t>priya@harborlights.example</t>
+  </si>
+  <si>
+    <t>+1 253 555 0177</t>
+  </si>
+  <si>
+    <t>https://linkedin.example/in/priya-natarajan</t>
+  </si>
+  <si>
+    <t>Dana Whitfield</t>
+  </si>
+  <si>
+    <t>Office Manager</t>
+  </si>
+  <si>
+    <t>dana@bluestemdental.example</t>
+  </si>
+  <si>
+    <t>+1 402 555 0126</t>
+  </si>
+  <si>
+    <t>Prefers afternoon calls</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hi Dana,
 thanks for the time this week.</t>
-  </si>
-  <si>
-    <t>P-005</t>
-  </si>
-  <si>
-    <t>Granite Peak Credit Union</t>
-  </si>
-  <si>
-    <t>Credit union</t>
-  </si>
-  <si>
-    <t>Boise, ID</t>
-  </si>
-  <si>
-    <t>granitepeakcu.example</t>
-  </si>
-  <si>
-    <t>Chose an incumbent</t>
-  </si>
-  <si>
-    <t>Conference</t>
-  </si>
-  <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>Signed a three-year deal with another vendor</t>
-  </si>
-  <si>
-    <t>P-006</t>
-  </si>
-  <si>
-    <t>Saltmarsh Marine Supply</t>
-  </si>
-  <si>
-    <t>Distributor</t>
-  </si>
-  <si>
-    <t>Mobile, AL</t>
-  </si>
-  <si>
-    <t>saltmarshmarine.example</t>
-  </si>
-  <si>
-    <t>Call Thursday</t>
-  </si>
-  <si>
-    <t>Seasonal push before spring</t>
-  </si>
-  <si>
-    <t>Paste new rows directly above this line, columns already in this order.</t>
-  </si>
-  <si>
-    <t>Prospect ID</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Contact type</t>
-  </si>
-  <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>LinkedIn</t>
-  </si>
-  <si>
-    <t>Last contacted</t>
-  </si>
-  <si>
-    <t>Last reply</t>
-  </si>
-  <si>
-    <t>Maya Okafor</t>
-  </si>
-  <si>
-    <t>Champion</t>
-  </si>
-  <si>
-    <t>Ms.</t>
-  </si>
-  <si>
-    <t>Plant Manager</t>
-  </si>
-  <si>
-    <t>maya.okafor@northwindfab.example</t>
-  </si>
-  <si>
-    <t>+1 937 555 0141</t>
-  </si>
-  <si>
-    <t>https://linkedin.example/in/maya-okafor</t>
-  </si>
-  <si>
-    <t>Met at the regional show</t>
-  </si>
-  <si>
-    <t>Tom Reyes</t>
-  </si>
-  <si>
-    <t>Technical Buyer</t>
-  </si>
-  <si>
-    <t>Mr.</t>
-  </si>
-  <si>
-    <t>IT Lead</t>
-  </si>
-  <si>
-    <t>tom.reyes@northwindfab.example</t>
-  </si>
-  <si>
-    <t>Priya Natarajan</t>
-  </si>
-  <si>
-    <t>Economic Buyer</t>
-  </si>
-  <si>
-    <t>VP Operations</t>
-  </si>
-  <si>
-    <t>priya@harborlights.example</t>
-  </si>
-  <si>
-    <t>+1 253 555 0177</t>
-  </si>
-  <si>
-    <t>https://linkedin.example/in/priya-natarajan</t>
-  </si>
-  <si>
-    <t>Dana Whitfield</t>
-  </si>
-  <si>
-    <t>Office Manager</t>
-  </si>
-  <si>
-    <t>dana@bluestemdental.example</t>
-  </si>
-  <si>
-    <t>+1 402 555 0126</t>
-  </si>
-  <si>
-    <t>Prefers afternoon calls</t>
   </si>
   <si>
     <t>Dr. Elise Marchetti</t>
@@ -1019,7 +1019,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <f>COUNTIF(Prospects!$Q$2:$Q$2000,"TRUE")</f>
+        <f>COUNTIF(Prospects!$P$2:$P$2000,"TRUE")</f>
         <v>1</v>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1061,12 +1061,11 @@
     <col min="12" max="12" width="20" style="5" customWidth="1"/>
     <col min="13" max="14" width="40" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="44" customWidth="1"/>
-    <col min="17" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="36" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>15</v>
       </c>
@@ -1113,21 +1112,18 @@
         <v>29</v>
       </c>
       <c r="P1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="6" t="s">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -1136,13 +1132,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>35</v>
-      </c>
-      <c r="G2" t="s">
-        <v>36</v>
       </c>
       <c r="H2" s="3">
         <v>420</v>
@@ -1151,27 +1147,26 @@
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="O2" t="s">
         <v>39</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" s="10"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="10"/>
-      <c r="R2" s="10"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>41</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -1180,13 +1175,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" t="s">
         <v>43</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>44</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
       </c>
       <c r="H3" s="3">
         <v>1100</v>
@@ -1195,27 +1190,26 @@
         <v>6</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="O3" t="s">
         <v>48</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" s="10"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
-      <c r="P3" s="10"/>
-      <c r="R3" s="10"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
@@ -1224,13 +1218,13 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>53</v>
-      </c>
-      <c r="G4" t="s">
-        <v>54</v>
       </c>
       <c r="H4" s="3">
         <v>260</v>
@@ -1240,21 +1234,20 @@
       </c>
       <c r="L4" s="5"/>
       <c r="M4" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N4" s="10"/>
       <c r="O4" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q4" s="10"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>56</v>
       </c>
-      <c r="P4" s="10"/>
-      <c r="R4" s="10"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -1263,13 +1256,13 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
         <v>59</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>60</v>
-      </c>
-      <c r="G5" t="s">
-        <v>61</v>
       </c>
       <c r="H5" s="3">
         <v>85</v>
@@ -1278,34 +1271,31 @@
         <v>7</v>
       </c>
       <c r="J5" t="s">
+        <v>61</v>
+      </c>
+      <c r="K5" t="s">
         <v>62</v>
-      </c>
-      <c r="K5" t="s">
-        <v>63</v>
       </c>
       <c r="L5" s="5">
         <v>46301.625</v>
       </c>
       <c r="M5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="O5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="10"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>65</v>
       </c>
-      <c r="O5" t="s">
-        <v>40</v>
-      </c>
-      <c r="P5" s="10" t="s">
+      <c r="B6" t="s">
         <v>66</v>
-      </c>
-      <c r="R5" s="10"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s">
-        <v>68</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
@@ -1314,13 +1304,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" t="s">
         <v>69</v>
-      </c>
-      <c r="F6" t="s">
-        <v>70</v>
-      </c>
-      <c r="G6" t="s">
-        <v>71</v>
       </c>
       <c r="H6" s="3">
         <v>190</v>
@@ -1331,25 +1321,24 @@
       <c r="L6" s="5"/>
       <c r="M6" s="10"/>
       <c r="N6" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="O6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P6" t="s">
         <v>72</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q6" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="P6" s="10"/>
-      <c r="Q6" t="s">
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>74</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="B7" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
@@ -1358,13 +1347,13 @@
         <v>6</v>
       </c>
       <c r="E7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" t="s">
         <v>78</v>
-      </c>
-      <c r="F7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G7" t="s">
-        <v>80</v>
       </c>
       <c r="H7" s="3">
         <v>60</v>
@@ -1373,26 +1362,25 @@
         <v>5</v>
       </c>
       <c r="J7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N7" s="10"/>
       <c r="O7" t="s">
-        <v>40</v>
-      </c>
-      <c r="P7" s="10"/>
-      <c r="R7" s="10"/>
+        <v>39</v>
+      </c>
+      <c r="Q7" s="10"/>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R7"/>
+  <autoFilter ref="A1:Q7"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="C2:C2000">
       <formula1>"Direct,Aggregator"</formula1>
@@ -1400,7 +1388,7 @@
     <dataValidation type="list" allowBlank="1" sqref="I2:I2000">
       <formula1>"Not contacted,Contacted,Replied,Meeting booked,Clinic held,Trial,Signed,Dead"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Q2:Q2000">
+    <dataValidation type="list" allowBlank="1" sqref="P2:P2000">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1415,7 +1403,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1431,140 +1419,146 @@
     <col min="11" max="11" width="14" style="12" customWidth="1"/>
     <col min="12" max="12" width="12" style="12" customWidth="1"/>
     <col min="13" max="13" width="40" customWidth="1"/>
+    <col min="14" max="14" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="L1" s="13" t="s">
         <v>92</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>94</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="s">
-        <v>33</v>
-      </c>
       <c r="C2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" t="s">
         <v>95</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" t="s">
         <v>96</v>
       </c>
-      <c r="E2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>97</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>98</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>99</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>100</v>
-      </c>
-      <c r="J2" t="s">
-        <v>101</v>
       </c>
       <c r="K2" s="12">
         <v>46287</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" t="s">
+        <v>101</v>
+      </c>
+      <c r="N2" s="10"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>103</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>104</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>105</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>106</v>
-      </c>
-      <c r="H3" t="s">
-        <v>107</v>
       </c>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3" s="10"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
       <c r="C4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" t="s">
         <v>108</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" t="s">
         <v>109</v>
       </c>
-      <c r="E4" t="s">
-        <v>74</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>110</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>111</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>112</v>
-      </c>
-      <c r="J4" t="s">
-        <v>113</v>
       </c>
       <c r="K4" s="12">
         <v>46290</v>
@@ -1572,50 +1566,54 @@
       <c r="L4" s="12">
         <v>46291</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4" s="10"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
         <v>57</v>
       </c>
-      <c r="B5" t="s">
-        <v>58</v>
-      </c>
       <c r="C5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" t="s">
         <v>114</v>
       </c>
-      <c r="D5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>115</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>116</v>
-      </c>
-      <c r="I5" t="s">
-        <v>117</v>
       </c>
       <c r="K5" s="12"/>
       <c r="L5" s="12"/>
       <c r="M5" t="s">
+        <v>117</v>
+      </c>
+      <c r="N5" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
         <v>57</v>
-      </c>
-      <c r="B6" t="s">
-        <v>58</v>
       </c>
       <c r="C6" t="s">
         <v>119</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
         <v>120</v>
@@ -1625,13 +1623,14 @@
       </c>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6" s="10"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
         <v>122</v>
@@ -1640,7 +1639,7 @@
         <v>123</v>
       </c>
       <c r="E7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G7" t="s">
         <v>124</v>
@@ -1650,13 +1649,14 @@
       </c>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7" s="10"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
         <v>126</v>
@@ -1665,7 +1665,7 @@
         <v>127</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G8" t="s">
         <v>128</v>
@@ -1680,9 +1680,10 @@
         <v>46295</v>
       </c>
       <c r="L8" s="12"/>
+      <c r="N8" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M8"/>
+  <autoFilter ref="A1:N8"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D2:D2000">
       <formula1>"Economic Buyer,Champion,Technical Buyer,End User,Influencer,Blocker,Gatekeeper,Channel"</formula1>

</xml_diff>

<commit_message>
Email source column on every campaign's contacts
New campaigns start with an Email source dropdown (Published, Reported,
Pattern, Verified) after Email, and import adds one to a Contacts tab
that lacks it. It stays an ordinary column the user can rename or delete.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/xlsx/fixtures/base-tracker.generated.xlsx
+++ b/src/xlsx/fixtures/base-tracker.generated.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="136">
   <si>
     <t>Pipeline summary</t>
   </si>
@@ -331,6 +331,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>Email source</t>
+  </si>
+  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -361,6 +364,9 @@
     <t>maya.okafor@northwindfab.example</t>
   </si>
   <si>
+    <t>Published</t>
+  </si>
+  <si>
     <t>+1 937 555 0141</t>
   </si>
   <si>
@@ -385,6 +391,9 @@
     <t>tom.reyes@northwindfab.example</t>
   </si>
   <si>
+    <t>Pattern</t>
+  </si>
+  <si>
     <t>Priya Natarajan</t>
   </si>
   <si>
@@ -397,6 +406,9 @@
     <t>priya@harborlights.example</t>
   </si>
   <si>
+    <t>Reported</t>
+  </si>
+  <si>
     <t>+1 253 555 0177</t>
   </si>
   <si>
@@ -410,6 +422,9 @@
   </si>
   <si>
     <t>dana@bluestemdental.example</t>
+  </si>
+  <si>
+    <t>Verified</t>
   </si>
   <si>
     <t>+1 402 555 0126</t>
@@ -1403,7 +1418,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1414,15 +1429,16 @@
     <col min="6" max="6" width="8" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="14" style="12" customWidth="1"/>
-    <col min="12" max="12" width="12" style="12" customWidth="1"/>
-    <col min="13" max="13" width="40" customWidth="1"/>
-    <col min="14" max="14" width="44" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="12" max="12" width="14" style="12" customWidth="1"/>
+    <col min="13" max="13" width="12" style="12" customWidth="1"/>
+    <col min="14" max="14" width="40" customWidth="1"/>
+    <col min="15" max="15" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>82</v>
       </c>
@@ -1453,20 +1469,23 @@
       <c r="J1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="6" t="s">
         <v>91</v>
       </c>
       <c r="L1" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="N1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1474,39 +1493,42 @@
         <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
         <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J2" t="s">
-        <v>100</v>
-      </c>
-      <c r="K2" s="12">
+        <v>101</v>
+      </c>
+      <c r="K2" t="s">
+        <v>102</v>
+      </c>
+      <c r="L2" s="12">
         <v>46287</v>
       </c>
-      <c r="L2" s="12"/>
-      <c r="M2" t="s">
-        <v>101</v>
-      </c>
-      <c r="N2" s="10"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M2" s="12"/>
+      <c r="N2" t="s">
+        <v>103</v>
+      </c>
+      <c r="O2" s="10"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1514,25 +1536,28 @@
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H3" t="s">
-        <v>106</v>
-      </c>
-      <c r="K3" s="12"/>
+        <v>108</v>
+      </c>
+      <c r="I3" t="s">
+        <v>109</v>
+      </c>
       <c r="L3" s="12"/>
-      <c r="N3" s="10"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M3" s="12"/>
+      <c r="O3" s="10"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -1540,35 +1565,38 @@
         <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
         <v>72</v>
       </c>
       <c r="G4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="J4" t="s">
-        <v>112</v>
-      </c>
-      <c r="K4" s="12">
+        <v>115</v>
+      </c>
+      <c r="K4" t="s">
+        <v>116</v>
+      </c>
+      <c r="L4" s="12">
         <v>46290</v>
       </c>
-      <c r="L4" s="12">
+      <c r="M4" s="12">
         <v>46291</v>
       </c>
-      <c r="N4" s="10"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O4" s="10"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -1576,33 +1604,36 @@
         <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5" t="s">
         <v>72</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I5" t="s">
-        <v>116</v>
-      </c>
-      <c r="K5" s="12"/>
+        <v>120</v>
+      </c>
+      <c r="J5" t="s">
+        <v>121</v>
+      </c>
       <c r="L5" s="12"/>
-      <c r="M5" t="s">
-        <v>117</v>
-      </c>
-      <c r="N5" s="10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M5" s="12"/>
+      <c r="N5" t="s">
+        <v>122</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>56</v>
       </c>
@@ -1610,22 +1641,22 @@
         <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>121</v>
-      </c>
-      <c r="K6" s="12"/>
+        <v>126</v>
+      </c>
       <c r="L6" s="12"/>
-      <c r="N6" s="10"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M6" s="12"/>
+      <c r="O6" s="10"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -1633,25 +1664,28 @@
         <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E7" t="s">
         <v>72</v>
       </c>
       <c r="G7" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="H7" t="s">
-        <v>125</v>
-      </c>
-      <c r="K7" s="12"/>
+        <v>130</v>
+      </c>
+      <c r="I7" t="s">
+        <v>100</v>
+      </c>
       <c r="L7" s="12"/>
-      <c r="N7" s="10"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M7" s="12"/>
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>74</v>
       </c>
@@ -1659,37 +1693,43 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
         <v>72</v>
       </c>
       <c r="G8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="H8" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="I8" t="s">
-        <v>130</v>
-      </c>
-      <c r="K8" s="12">
+        <v>109</v>
+      </c>
+      <c r="J8" t="s">
+        <v>135</v>
+      </c>
+      <c r="L8" s="12">
         <v>46295</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="N8" s="10"/>
+      <c r="M8" s="12"/>
+      <c r="O8" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N8"/>
-  <dataValidations count="2">
+  <autoFilter ref="A1:O8"/>
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="D2:D2000">
       <formula1>"Economic Buyer,Champion,Technical Buyer,End User,Influencer,Blocker,Gatekeeper,Channel"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E2:E2000">
       <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I2000">
+      <formula1>"Published,Reported,Pattern,Verified"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>